<commit_message>
feat(surveys): Developer Survey options in EN, PT-BR and ES, Spanish survey outputs, no dashes
survey-devs/options.json maps the options of the three banks (and older
Portuguese options with dashes) to the same canonical option before
scoring, so results do not depend on the form language; the insights show
options in the report language. The survey scripts and the wizard
auto-fill now write Spanish. Survey banks, templates and docs drop em and
en dashes; generated survey Markdown is lint-clean with email links. Also
fixes a missing PT-BR text key in calcular_maturidade.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
Copilot-Session: f9fd4a8a-033c-4218-b2f1-2c8da428242c
</commit_message>
<xml_diff>
--- a/survey-devs/template-export-forms-devs.xlsx
+++ b/survey-devs/template-export-forms-devs.xlsx
@@ -639,12 +639,12 @@
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>S3-Q3: Conhece o GitHub Copilot Coding Agent (sucessor do Workspace, GA set/2025 — assigna issue e abre PR sozinho)?</t>
+          <t>S3-Q3: Conhece o GitHub Copilot Coding Agent (sucessor do Workspace, GA set/2025: assigna issue e abre PR sozinho)?</t>
         </is>
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>S3-Q4: Conhece Copilot Spaces (contexto compartilhado — substituiu Knowledge Bases)?</t>
+          <t>S3-Q4: Conhece Copilot Spaces (contexto compartilhado: substituiu Knowledge Bases)?</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
@@ -654,7 +654,7 @@
       </c>
       <c r="AA1" s="1" t="inlineStr">
         <is>
-          <t>S3-Q6: Conhece MCP (Model Context Protocol) — padrão para agentes consumirem tools/contexto?</t>
+          <t>S3-Q6: Conhece MCP (Model Context Protocol): padrão para agentes consumirem tools/contexto?</t>
         </is>
       </c>
       <c r="AB1" s="1" t="inlineStr">
@@ -664,12 +664,12 @@
       </c>
       <c r="AC1" s="1" t="inlineStr">
         <is>
-          <t>S4-Q1: Você pratica TDD (Test-Driven Development) com IA — escrever teste primeiro com Copilot?</t>
+          <t>S4-Q1: Você pratica TDD (Test-Driven Development) com IA: escrever teste primeiro com Copilot?</t>
         </is>
       </c>
       <c r="AD1" s="1" t="inlineStr">
         <is>
-          <t>S4-Q2: Você pratica SDD (Spec-Driven Development) — escrever spec → IA gera código?</t>
+          <t>S4-Q2: Você pratica SDD (Spec-Driven Development): escrever spec → IA gera código?</t>
         </is>
       </c>
       <c r="AE1" s="1" t="inlineStr">
@@ -699,7 +699,7 @@
       </c>
       <c r="AJ1" s="1" t="inlineStr">
         <is>
-          <t>S4-Q8: Onboarding em projeto novo — você usa IA (com Copilot Spaces ou similar) para entender a base de código?</t>
+          <t>S4-Q8: Onboarding em projeto novo: você usa IA (com Copilot Spaces ou similar) para entender a base de código?</t>
         </is>
       </c>
       <c r="AK1" s="1" t="inlineStr">
@@ -724,7 +724,7 @@
       </c>
       <c r="AO1" s="1" t="inlineStr">
         <is>
-          <t>S5-Q4: Você conhece o conceito de 'skill' (SKILL.md ou equivalente — bloco reutilizável de instruções)?</t>
+          <t>S5-Q4: Você conhece o conceito de 'skill' (SKILL.md ou equivalente: bloco reutilizável de instruções)?</t>
         </is>
       </c>
       <c r="AP1" s="1" t="inlineStr">
@@ -734,7 +734,7 @@
       </c>
       <c r="AQ1" s="1" t="inlineStr">
         <is>
-          <t>S5-Q6: Conhece A2A (Agent-to-Agent protocol) — agentes comunicando entre si?</t>
+          <t>S5-Q6: Conhece A2A (Agent-to-Agent protocol): agentes comunicando entre si?</t>
         </is>
       </c>
       <c r="AR1" s="1" t="inlineStr">
@@ -879,7 +879,7 @@
       </c>
       <c r="BT1" s="1" t="inlineStr">
         <is>
-          <t>S8-Q9: Sua org tem permissões JIT (Just-In-Time) para agents — vs. permissões persistentes?</t>
+          <t>S8-Q9: Sua org tem permissões JIT (Just-In-Time) para agents: vs. permissões persistentes?</t>
         </is>
       </c>
       <c r="BU1" s="1" t="inlineStr">
@@ -889,7 +889,7 @@
       </c>
       <c r="BV1" s="1" t="inlineStr">
         <is>
-          <t>S8-Q11: Sua org tem AUDIT LOGS de uso do Copilot/agentes IA — incluindo decisões autônomas de agents?</t>
+          <t>S8-Q11: Sua org tem AUDIT LOGS de uso do Copilot/agentes IA: incluindo decisões autônomas de agents?</t>
         </is>
       </c>
       <c r="BW1" s="1" t="inlineStr">
@@ -984,7 +984,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Sim — Copilot Pro (individual)</t>
+          <t>Sim, Copilot Pro (individual)</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -1099,7 +1099,7 @@
       </c>
       <c r="AJ2" t="inlineStr">
         <is>
-          <t>Sempre — primeira coisa que faço</t>
+          <t>Sempre, primeira coisa que faço</t>
         </is>
       </c>
       <c r="AK2" t="inlineStr">
@@ -1109,12 +1109,12 @@
       </c>
       <c r="AL2" t="inlineStr">
         <is>
-          <t>Sim — vagamente</t>
+          <t>Sim, vagamente</t>
         </is>
       </c>
       <c r="AM2" t="inlineStr">
         <is>
-          <t>Sim — uso conscientemente</t>
+          <t>Sim, uso conscientemente</t>
         </is>
       </c>
       <c r="AN2" t="inlineStr">
@@ -1129,7 +1129,7 @@
       </c>
       <c r="AP2" t="inlineStr">
         <is>
-          <t>Sim — uma ou duas</t>
+          <t>Sim, uma ou duas</t>
         </is>
       </c>
       <c r="AQ2" t="inlineStr">
@@ -1154,7 +1154,7 @@
       </c>
       <c r="AU2" t="inlineStr">
         <is>
-          <t>Sempre — tenho test suite para meus agents</t>
+          <t>Sempre, tenho test suite para meus agents</t>
         </is>
       </c>
       <c r="AV2" t="inlineStr">
@@ -1184,7 +1184,7 @@
       </c>
       <c r="BA2" t="inlineStr">
         <is>
-          <t>Sim — repo dedicado</t>
+          <t>Sim, repo dedicado</t>
         </is>
       </c>
       <c r="BB2" t="inlineStr">
@@ -1199,12 +1199,12 @@
       </c>
       <c r="BD2" t="inlineStr">
         <is>
-          <t>Sim — eu sou</t>
+          <t>Sim, eu sou</t>
         </is>
       </c>
       <c r="BE2" t="inlineStr">
         <is>
-          <t>Sim — ativo (&gt;5 mensagens/semana)</t>
+          <t>Sim, ativo (&gt;5 mensagens/semana)</t>
         </is>
       </c>
       <c r="BF2" t="inlineStr">
@@ -1234,12 +1234,12 @@
       </c>
       <c r="BK2" t="inlineStr">
         <is>
-          <t>Às vezes — pessoalmente</t>
+          <t>Às vezes, pessoalmente</t>
         </is>
       </c>
       <c r="BL2" t="inlineStr">
         <is>
-          <t>Sim — mas pouco clara</t>
+          <t>Sim, mas pouco clara</t>
         </is>
       </c>
       <c r="BM2" t="inlineStr">
@@ -1259,12 +1259,12 @@
       </c>
       <c r="BP2" t="inlineStr">
         <is>
-          <t>Sim — opcional</t>
+          <t>Sim, opcional</t>
         </is>
       </c>
       <c r="BQ2" t="inlineStr">
         <is>
-          <t>Sim — manual quando solicitado</t>
+          <t>Sim, manual quando solicitado</t>
         </is>
       </c>
       <c r="BR2" t="inlineStr">
@@ -1274,27 +1274,27 @@
       </c>
       <c r="BS2" t="inlineStr">
         <is>
-          <t>Sempre — escopo + red-lines documentados</t>
+          <t>Sempre, escopo + red-lines documentados</t>
         </is>
       </c>
       <c r="BT2" t="inlineStr">
         <is>
-          <t>Sim — JIT obrigatório para agents</t>
+          <t>Sim, JIT obrigatório para agents</t>
         </is>
       </c>
       <c r="BU2" t="inlineStr">
         <is>
-          <t>Sim — alerta mas não bloqueia</t>
+          <t>Sim, alerta mas não bloqueia</t>
         </is>
       </c>
       <c r="BV2" t="inlineStr">
         <is>
-          <t>Sim — logs ativos e revisados</t>
+          <t>Sim, logs ativos e revisados</t>
         </is>
       </c>
       <c r="BW2" t="inlineStr">
         <is>
-          <t>Sim — treinamento obrigatório anual</t>
+          <t>Sim, treinamento obrigatório anual</t>
         </is>
       </c>
       <c r="BX2" t="inlineStr">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="CB2" t="inlineStr">
         <is>
-          <t>Sim — quero ver</t>
+          <t>Sim, quero ver</t>
         </is>
       </c>
     </row>
@@ -1394,7 +1394,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Plan / Vision; Agent (autônomo no IDE, executa tasks); Não uso o Chat — só completion inline; Ask (responder perguntas)</t>
+          <t>Plan / Vision; Agent (autônomo no IDE, executa tasks); Não uso o Chat, só completion inline; Ask (responder perguntas)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -1529,7 +1529,7 @@
       </c>
       <c r="AP3" t="inlineStr">
         <is>
-          <t>Sim — uma ou duas</t>
+          <t>Sim, uma ou duas</t>
         </is>
       </c>
       <c r="AQ3" t="inlineStr">
@@ -1554,7 +1554,7 @@
       </c>
       <c r="AU3" t="inlineStr">
         <is>
-          <t>Às vezes — só sanity check</t>
+          <t>Às vezes, só sanity check</t>
         </is>
       </c>
       <c r="AV3" t="inlineStr">
@@ -1584,7 +1584,7 @@
       </c>
       <c r="BA3" t="inlineStr">
         <is>
-          <t>Sim — Copilot Space compartilhado</t>
+          <t>Sim, Copilot Space compartilhado</t>
         </is>
       </c>
       <c r="BB3" t="inlineStr">
@@ -1604,7 +1604,7 @@
       </c>
       <c r="BE3" t="inlineStr">
         <is>
-          <t>Sim — ativo (&gt;5 mensagens/semana)</t>
+          <t>Sim, ativo (&gt;5 mensagens/semana)</t>
         </is>
       </c>
       <c r="BF3" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="BL3" t="inlineStr">
         <is>
-          <t>Sim — mas pouco clara</t>
+          <t>Sim, mas pouco clara</t>
         </is>
       </c>
       <c r="BM3" t="inlineStr">
@@ -1659,17 +1659,17 @@
       </c>
       <c r="BP3" t="inlineStr">
         <is>
-          <t>Sim — gate obrigatório no PR</t>
+          <t>Sim, gate obrigatório no PR</t>
         </is>
       </c>
       <c r="BQ3" t="inlineStr">
         <is>
-          <t>Sim — automatizado</t>
+          <t>Sim, automatizado</t>
         </is>
       </c>
       <c r="BR3" t="inlineStr">
         <is>
-          <t>Sim — review obrigatório por outro humano + scanner</t>
+          <t>Sim, review obrigatório por outro humano + scanner</t>
         </is>
       </c>
       <c r="BS3" t="inlineStr">
@@ -1684,7 +1684,7 @@
       </c>
       <c r="BU3" t="inlineStr">
         <is>
-          <t>Sim — bloqueia ativamente</t>
+          <t>Sim, bloqueia ativamente</t>
         </is>
       </c>
       <c r="BV3" t="inlineStr">
@@ -1694,7 +1694,7 @@
       </c>
       <c r="BW3" t="inlineStr">
         <is>
-          <t>Sim — uma vez (no onboarding)</t>
+          <t>Sim, uma vez (no onboarding)</t>
         </is>
       </c>
       <c r="BX3" t="inlineStr">
@@ -1784,7 +1784,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Sim — Copilot Enterprise</t>
+          <t>Sim, Copilot Enterprise</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -1899,7 +1899,7 @@
       </c>
       <c r="AJ4" t="inlineStr">
         <is>
-          <t>Sempre — primeira coisa que faço</t>
+          <t>Sempre, primeira coisa que faço</t>
         </is>
       </c>
       <c r="AK4" t="inlineStr">
@@ -1909,7 +1909,7 @@
       </c>
       <c r="AL4" t="inlineStr">
         <is>
-          <t>Sim — explico claramente</t>
+          <t>Sim, explico claramente</t>
         </is>
       </c>
       <c r="AM4" t="inlineStr">
@@ -1929,7 +1929,7 @@
       </c>
       <c r="AP4" t="inlineStr">
         <is>
-          <t>Sim — várias</t>
+          <t>Sim, várias</t>
         </is>
       </c>
       <c r="AQ4" t="inlineStr">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="AU4" t="inlineStr">
         <is>
-          <t>Sempre — tenho test suite para meus agents</t>
+          <t>Sempre, tenho test suite para meus agents</t>
         </is>
       </c>
       <c r="AV4" t="inlineStr">
@@ -1984,7 +1984,7 @@
       </c>
       <c r="BA4" t="inlineStr">
         <is>
-          <t>Sim — wiki/Confluence</t>
+          <t>Sim, wiki/Confluence</t>
         </is>
       </c>
       <c r="BB4" t="inlineStr">
@@ -1999,12 +1999,12 @@
       </c>
       <c r="BD4" t="inlineStr">
         <is>
-          <t>Sim — eu sou</t>
+          <t>Sim, eu sou</t>
         </is>
       </c>
       <c r="BE4" t="inlineStr">
         <is>
-          <t>Sim — ativo (&gt;5 mensagens/semana)</t>
+          <t>Sim, ativo (&gt;5 mensagens/semana)</t>
         </is>
       </c>
       <c r="BF4" t="inlineStr">
@@ -2019,7 +2019,7 @@
       </c>
       <c r="BH4" t="inlineStr">
         <is>
-          <t>Nunca — sempre reviso</t>
+          <t>Nunca, sempre reviso</t>
         </is>
       </c>
       <c r="BI4" t="inlineStr">
@@ -2039,7 +2039,7 @@
       </c>
       <c r="BL4" t="inlineStr">
         <is>
-          <t>Sim — mas pouco clara</t>
+          <t>Sim, mas pouco clara</t>
         </is>
       </c>
       <c r="BM4" t="inlineStr">
@@ -2059,12 +2059,12 @@
       </c>
       <c r="BP4" t="inlineStr">
         <is>
-          <t>Sim — gate obrigatório no PR</t>
+          <t>Sim, gate obrigatório no PR</t>
         </is>
       </c>
       <c r="BQ4" t="inlineStr">
         <is>
-          <t>Sim — automatizado</t>
+          <t>Sim, automatizado</t>
         </is>
       </c>
       <c r="BR4" t="inlineStr">
@@ -2084,7 +2084,7 @@
       </c>
       <c r="BU4" t="inlineStr">
         <is>
-          <t>Sim — alerta mas não bloqueia</t>
+          <t>Sim, alerta mas não bloqueia</t>
         </is>
       </c>
       <c r="BV4" t="inlineStr">
@@ -2094,7 +2094,7 @@
       </c>
       <c r="BW4" t="inlineStr">
         <is>
-          <t>Sim — uma vez (no onboarding)</t>
+          <t>Sim, uma vez (no onboarding)</t>
         </is>
       </c>
       <c r="BX4" t="inlineStr">
@@ -2184,7 +2184,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Sim — Copilot Business</t>
+          <t>Sim, Copilot Business</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -2194,7 +2194,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Plan / Vision; Não uso o Chat — só completion inline; Copilot Coding Agent (autônomo no GitHub.com — assigna issue, abre PR sozinho)</t>
+          <t>Plan / Vision; Não uso o Chat, só completion inline; Copilot Coding Agent (autônomo no GitHub.com, assigna issue, abre PR sozinho)</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -2299,7 +2299,7 @@
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
-          <t>Sempre — primeira coisa que faço</t>
+          <t>Sempre, primeira coisa que faço</t>
         </is>
       </c>
       <c r="AK5" t="inlineStr">
@@ -2309,12 +2309,12 @@
       </c>
       <c r="AL5" t="inlineStr">
         <is>
-          <t>Sim — vagamente</t>
+          <t>Sim, vagamente</t>
         </is>
       </c>
       <c r="AM5" t="inlineStr">
         <is>
-          <t>Sim — uso conscientemente</t>
+          <t>Sim, uso conscientemente</t>
         </is>
       </c>
       <c r="AN5" t="inlineStr">
@@ -2329,7 +2329,7 @@
       </c>
       <c r="AP5" t="inlineStr">
         <is>
-          <t>Sim — várias</t>
+          <t>Sim, várias</t>
         </is>
       </c>
       <c r="AQ5" t="inlineStr">
@@ -2349,12 +2349,12 @@
       </c>
       <c r="AT5" t="inlineStr">
         <is>
-          <t>Sim — adoto explicitamente</t>
+          <t>Sim, adoto explicitamente</t>
         </is>
       </c>
       <c r="AU5" t="inlineStr">
         <is>
-          <t>Sempre — tenho test suite para meus agents</t>
+          <t>Sempre, tenho test suite para meus agents</t>
         </is>
       </c>
       <c r="AV5" t="inlineStr">
@@ -2384,7 +2384,7 @@
       </c>
       <c r="BA5" t="inlineStr">
         <is>
-          <t>Sim — Copilot Space compartilhado</t>
+          <t>Sim, Copilot Space compartilhado</t>
         </is>
       </c>
       <c r="BB5" t="inlineStr">
@@ -2399,12 +2399,12 @@
       </c>
       <c r="BD5" t="inlineStr">
         <is>
-          <t>Sim — eu sou</t>
+          <t>Sim, eu sou</t>
         </is>
       </c>
       <c r="BE5" t="inlineStr">
         <is>
-          <t>Sim — ativo (&gt;5 mensagens/semana)</t>
+          <t>Sim, ativo (&gt;5 mensagens/semana)</t>
         </is>
       </c>
       <c r="BF5" t="inlineStr">
@@ -2434,7 +2434,7 @@
       </c>
       <c r="BK5" t="inlineStr">
         <is>
-          <t>Frequentemente — em canal compartilhado</t>
+          <t>Frequentemente, em canal compartilhado</t>
         </is>
       </c>
       <c r="BL5" t="inlineStr">
@@ -2459,17 +2459,17 @@
       </c>
       <c r="BP5" t="inlineStr">
         <is>
-          <t>Sim — opcional</t>
+          <t>Sim, opcional</t>
         </is>
       </c>
       <c r="BQ5" t="inlineStr">
         <is>
-          <t>Sim — manual quando solicitado</t>
+          <t>Sim, manual quando solicitado</t>
         </is>
       </c>
       <c r="BR5" t="inlineStr">
         <is>
-          <t>Sim — review obrigatório por outro humano + scanner</t>
+          <t>Sim, review obrigatório por outro humano + scanner</t>
         </is>
       </c>
       <c r="BS5" t="inlineStr">
@@ -2479,12 +2479,12 @@
       </c>
       <c r="BT5" t="inlineStr">
         <is>
-          <t>Sim — opcional</t>
+          <t>Sim, opcional</t>
         </is>
       </c>
       <c r="BU5" t="inlineStr">
         <is>
-          <t>Sim — alerta mas não bloqueia</t>
+          <t>Sim, alerta mas não bloqueia</t>
         </is>
       </c>
       <c r="BV5" t="inlineStr">
@@ -2494,7 +2494,7 @@
       </c>
       <c r="BW5" t="inlineStr">
         <is>
-          <t>Sim — uma vez (no onboarding)</t>
+          <t>Sim, uma vez (no onboarding)</t>
         </is>
       </c>
       <c r="BX5" t="inlineStr">
@@ -2584,7 +2584,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Sim — Copilot Pro (individual)</t>
+          <t>Sim, Copilot Pro (individual)</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -2709,12 +2709,12 @@
       </c>
       <c r="AL6" t="inlineStr">
         <is>
-          <t>Sim — explico claramente</t>
+          <t>Sim, explico claramente</t>
         </is>
       </c>
       <c r="AM6" t="inlineStr">
         <is>
-          <t>Sim — uso conscientemente</t>
+          <t>Sim, uso conscientemente</t>
         </is>
       </c>
       <c r="AN6" t="inlineStr">
@@ -2729,7 +2729,7 @@
       </c>
       <c r="AP6" t="inlineStr">
         <is>
-          <t>Sim — uma ou duas</t>
+          <t>Sim, uma ou duas</t>
         </is>
       </c>
       <c r="AQ6" t="inlineStr">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="AU6" t="inlineStr">
         <is>
-          <t>Frequentemente — manual mas sistemático</t>
+          <t>Frequentemente, manual mas sistemático</t>
         </is>
       </c>
       <c r="AV6" t="inlineStr">
@@ -2784,7 +2784,7 @@
       </c>
       <c r="BA6" t="inlineStr">
         <is>
-          <t>Sim — wiki/Confluence</t>
+          <t>Sim, wiki/Confluence</t>
         </is>
       </c>
       <c r="BB6" t="inlineStr">
@@ -2799,12 +2799,12 @@
       </c>
       <c r="BD6" t="inlineStr">
         <is>
-          <t>Sim — outra pessoa</t>
+          <t>Sim, outra pessoa</t>
         </is>
       </c>
       <c r="BE6" t="inlineStr">
         <is>
-          <t>Sim — pouco ativo</t>
+          <t>Sim, pouco ativo</t>
         </is>
       </c>
       <c r="BF6" t="inlineStr">
@@ -2834,12 +2834,12 @@
       </c>
       <c r="BK6" t="inlineStr">
         <is>
-          <t>Às vezes — pessoalmente</t>
+          <t>Às vezes, pessoalmente</t>
         </is>
       </c>
       <c r="BL6" t="inlineStr">
         <is>
-          <t>Sim — política formal e clara</t>
+          <t>Sim, política formal e clara</t>
         </is>
       </c>
       <c r="BM6" t="inlineStr">
@@ -2859,32 +2859,32 @@
       </c>
       <c r="BP6" t="inlineStr">
         <is>
-          <t>Sim — opcional</t>
+          <t>Sim, opcional</t>
         </is>
       </c>
       <c r="BQ6" t="inlineStr">
         <is>
-          <t>Sim — automatizado</t>
+          <t>Sim, automatizado</t>
         </is>
       </c>
       <c r="BR6" t="inlineStr">
         <is>
-          <t>Sim — review obrigatório por outro humano + scanner</t>
+          <t>Sim, review obrigatório por outro humano + scanner</t>
         </is>
       </c>
       <c r="BS6" t="inlineStr">
         <is>
-          <t>Sempre — escopo + red-lines documentados</t>
+          <t>Sempre, escopo + red-lines documentados</t>
         </is>
       </c>
       <c r="BT6" t="inlineStr">
         <is>
-          <t>Sim — opcional</t>
+          <t>Sim, opcional</t>
         </is>
       </c>
       <c r="BU6" t="inlineStr">
         <is>
-          <t>Sim — alerta mas não bloqueia</t>
+          <t>Sim, alerta mas não bloqueia</t>
         </is>
       </c>
       <c r="BV6" t="inlineStr">
@@ -2894,7 +2894,7 @@
       </c>
       <c r="BW6" t="inlineStr">
         <is>
-          <t>Sim — uma vez (no onboarding)</t>
+          <t>Sim, uma vez (no onboarding)</t>
         </is>
       </c>
       <c r="BX6" t="inlineStr">
@@ -2919,7 +2919,7 @@
       </c>
       <c r="CB6" t="inlineStr">
         <is>
-          <t>Sim — quero ver</t>
+          <t>Sim, quero ver</t>
         </is>
       </c>
     </row>
@@ -2947,9 +2947,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -2964,9 +2962,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
@@ -3016,9 +3012,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr"/>
-    </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
@@ -3061,9 +3055,7 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr"/>
-    </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>

</xml_diff>